<commit_message>
PEPI: incrustar valores en cache en el Excel (formulas + valores)
Las celdas de amortizacion, flujos e indicadores conservan sus formulas
vivas y ahora ademas guardan el valor calculado en cache, para que se
vean correctamente en cualquier visor (GitHub, Google Sheets, Excel en
vista protegida) que no recalcula automaticamente. Se anade fullCalcOnLoad.
</commit_message>
<xml_diff>
--- a/Proyectos/PEPI/Solucion/MODELO FINANCIERO PEPI.xlsx
+++ b/Proyectos/PEPI/Solucion/MODELO FINANCIERO PEPI.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno de Caudal" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amortizacion Deuda" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flujos de Caja" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Diseno de Caudal" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Supuestos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Amortizacion Deuda" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Flujos de Caja" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Indicadores" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Riesgos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -578,6 +578,7 @@
       </c>
       <c r="B6" s="4">
         <f>B4*B5</f>
+        <v>10200.0</v>
         <v/>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -639,6 +640,7 @@
       </c>
       <c r="B10" s="4">
         <f>B6*(1+B8)^(B7-2018)</f>
+        <v>10956.7877</v>
         <v/>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -655,6 +657,7 @@
       </c>
       <c r="B11" s="4">
         <f>B10*(1+B8)^B9</f>
+        <v>14763.728817</v>
         <v/>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -701,6 +704,7 @@
       </c>
       <c r="B14" s="4">
         <f>B12/(1-B13)</f>
+        <v>186.666667</v>
         <v/>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -747,6 +751,7 @@
       </c>
       <c r="B17" s="4">
         <f>B11*B14/86400</f>
+        <v>31.896945</v>
         <v/>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -763,6 +768,7 @@
       </c>
       <c r="B18" s="4">
         <f>B17*B15</f>
+        <v>41.466028</v>
         <v/>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -779,6 +785,7 @@
       </c>
       <c r="B19" s="4">
         <f>B18*B16</f>
+        <v>66.345646</v>
         <v/>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -923,6 +930,7 @@
       </c>
       <c r="B8" s="8">
         <f>B4*B5</f>
+        <v>15976.8</v>
         <v/>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -939,6 +947,7 @@
       </c>
       <c r="B9" s="8">
         <f>B4*B6</f>
+        <v>1997.1</v>
         <v/>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -955,6 +964,7 @@
       </c>
       <c r="B10" s="8">
         <f>B4*B7</f>
+        <v>1997.1</v>
         <v/>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1151,6 +1161,7 @@
       </c>
       <c r="B23" s="8">
         <f>B4/B16</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -1167,6 +1178,7 @@
       </c>
       <c r="B24" s="8">
         <f>B9*B11/(1-(1+B11)^(-B15))</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -1183,6 +1195,7 @@
       </c>
       <c r="B25" s="10">
         <f>B5*B13+B7*B12+B6*B11*(1-B14)</f>
+        <v>0.09315</v>
         <v/>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -1261,22 +1274,27 @@
       </c>
       <c r="B3" s="8">
         <f>Supuestos!$B$9</f>
+        <v>1997.1</v>
         <v/>
       </c>
       <c r="C3" s="8">
         <f>IF(A3&lt;=Supuestos!$B$15,B3*Supuestos!$B$11,0)</f>
+        <v>219.681</v>
         <v/>
       </c>
       <c r="D3" s="8">
         <f>E3-C3</f>
+        <v>119.42943</v>
         <v/>
       </c>
       <c r="E3" s="8">
         <f>IF(A3&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F3" s="8">
         <f>B3-D3</f>
+        <v>1877.67057</v>
         <v/>
       </c>
     </row>
@@ -1286,22 +1304,27 @@
       </c>
       <c r="B4" s="12">
         <f>F3</f>
+        <v>1877.67057</v>
         <v/>
       </c>
       <c r="C4" s="12">
         <f>IF(A4&lt;=Supuestos!$B$15,B4*Supuestos!$B$11,0)</f>
+        <v>206.543763</v>
         <v/>
       </c>
       <c r="D4" s="12">
         <f>E4-C4</f>
+        <v>132.566667</v>
         <v/>
       </c>
       <c r="E4" s="12">
         <f>IF(A4&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F4" s="12">
         <f>B4-D4</f>
+        <v>1745.103903</v>
         <v/>
       </c>
     </row>
@@ -1311,22 +1334,27 @@
       </c>
       <c r="B5" s="8">
         <f>F4</f>
+        <v>1745.103903</v>
         <v/>
       </c>
       <c r="C5" s="8">
         <f>IF(A5&lt;=Supuestos!$B$15,B5*Supuestos!$B$11,0)</f>
+        <v>191.961429</v>
         <v/>
       </c>
       <c r="D5" s="8">
         <f>E5-C5</f>
+        <v>147.149001</v>
         <v/>
       </c>
       <c r="E5" s="8">
         <f>IF(A5&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F5" s="8">
         <f>B5-D5</f>
+        <v>1597.954902</v>
         <v/>
       </c>
     </row>
@@ -1336,22 +1364,27 @@
       </c>
       <c r="B6" s="12">
         <f>F5</f>
+        <v>1597.954902</v>
         <v/>
       </c>
       <c r="C6" s="12">
         <f>IF(A6&lt;=Supuestos!$B$15,B6*Supuestos!$B$11,0)</f>
+        <v>175.775039</v>
         <v/>
       </c>
       <c r="D6" s="12">
         <f>E6-C6</f>
+        <v>163.335391</v>
         <v/>
       </c>
       <c r="E6" s="12">
         <f>IF(A6&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F6" s="12">
         <f>B6-D6</f>
+        <v>1434.619511</v>
         <v/>
       </c>
     </row>
@@ -1361,22 +1394,27 @@
       </c>
       <c r="B7" s="8">
         <f>F6</f>
+        <v>1434.619511</v>
         <v/>
       </c>
       <c r="C7" s="8">
         <f>IF(A7&lt;=Supuestos!$B$15,B7*Supuestos!$B$11,0)</f>
+        <v>157.808146</v>
         <v/>
       </c>
       <c r="D7" s="8">
         <f>E7-C7</f>
+        <v>181.302284</v>
         <v/>
       </c>
       <c r="E7" s="8">
         <f>IF(A7&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F7" s="8">
         <f>B7-D7</f>
+        <v>1253.317227</v>
         <v/>
       </c>
     </row>
@@ -1386,22 +1424,27 @@
       </c>
       <c r="B8" s="12">
         <f>F7</f>
+        <v>1253.317227</v>
         <v/>
       </c>
       <c r="C8" s="12">
         <f>IF(A8&lt;=Supuestos!$B$15,B8*Supuestos!$B$11,0)</f>
+        <v>137.864895</v>
         <v/>
       </c>
       <c r="D8" s="12">
         <f>E8-C8</f>
+        <v>201.245535</v>
         <v/>
       </c>
       <c r="E8" s="12">
         <f>IF(A8&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F8" s="12">
         <f>B8-D8</f>
+        <v>1052.071692</v>
         <v/>
       </c>
     </row>
@@ -1411,22 +1454,27 @@
       </c>
       <c r="B9" s="8">
         <f>F8</f>
+        <v>1052.071692</v>
         <v/>
       </c>
       <c r="C9" s="8">
         <f>IF(A9&lt;=Supuestos!$B$15,B9*Supuestos!$B$11,0)</f>
+        <v>115.727886</v>
         <v/>
       </c>
       <c r="D9" s="8">
         <f>E9-C9</f>
+        <v>223.382544</v>
         <v/>
       </c>
       <c r="E9" s="8">
         <f>IF(A9&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F9" s="8">
         <f>B9-D9</f>
+        <v>828.689148</v>
         <v/>
       </c>
     </row>
@@ -1436,22 +1484,27 @@
       </c>
       <c r="B10" s="12">
         <f>F9</f>
+        <v>828.689148</v>
         <v/>
       </c>
       <c r="C10" s="12">
         <f>IF(A10&lt;=Supuestos!$B$15,B10*Supuestos!$B$11,0)</f>
+        <v>91.155806</v>
         <v/>
       </c>
       <c r="D10" s="12">
         <f>E10-C10</f>
+        <v>247.954624</v>
         <v/>
       </c>
       <c r="E10" s="12">
         <f>IF(A10&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F10" s="12">
         <f>B10-D10</f>
+        <v>580.734524</v>
         <v/>
       </c>
     </row>
@@ -1461,22 +1514,27 @@
       </c>
       <c r="B11" s="8">
         <f>F10</f>
+        <v>580.734524</v>
         <v/>
       </c>
       <c r="C11" s="8">
         <f>IF(A11&lt;=Supuestos!$B$15,B11*Supuestos!$B$11,0)</f>
+        <v>63.880798</v>
         <v/>
       </c>
       <c r="D11" s="8">
         <f>E11-C11</f>
+        <v>275.229632</v>
         <v/>
       </c>
       <c r="E11" s="8">
         <f>IF(A11&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F11" s="8">
         <f>B11-D11</f>
+        <v>305.504892</v>
         <v/>
       </c>
     </row>
@@ -1486,22 +1544,27 @@
       </c>
       <c r="B12" s="12">
         <f>F11</f>
+        <v>305.504892</v>
         <v/>
       </c>
       <c r="C12" s="12">
         <f>IF(A12&lt;=Supuestos!$B$15,B12*Supuestos!$B$11,0)</f>
+        <v>33.605538</v>
         <v/>
       </c>
       <c r="D12" s="12">
         <f>E12-C12</f>
+        <v>305.504892</v>
         <v/>
       </c>
       <c r="E12" s="12">
         <f>IF(A12&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>339.11043</v>
         <v/>
       </c>
       <c r="F12" s="12">
         <f>B12-D12</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1511,22 +1574,27 @@
       </c>
       <c r="B13" s="8">
         <f>F12</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C13" s="8">
         <f>IF(A13&lt;=Supuestos!$B$15,B13*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D13" s="8">
         <f>E13-C13</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E13" s="8">
         <f>IF(A13&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F13" s="8">
         <f>B13-D13</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1536,22 +1604,27 @@
       </c>
       <c r="B14" s="12">
         <f>F13</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C14" s="12">
         <f>IF(A14&lt;=Supuestos!$B$15,B14*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D14" s="12">
         <f>E14-C14</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E14" s="12">
         <f>IF(A14&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F14" s="12">
         <f>B14-D14</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1561,22 +1634,27 @@
       </c>
       <c r="B15" s="8">
         <f>F14</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C15" s="8">
         <f>IF(A15&lt;=Supuestos!$B$15,B15*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D15" s="8">
         <f>E15-C15</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E15" s="8">
         <f>IF(A15&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F15" s="8">
         <f>B15-D15</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1586,22 +1664,27 @@
       </c>
       <c r="B16" s="12">
         <f>F15</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C16" s="12">
         <f>IF(A16&lt;=Supuestos!$B$15,B16*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D16" s="12">
         <f>E16-C16</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E16" s="12">
         <f>IF(A16&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F16" s="12">
         <f>B16-D16</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1611,22 +1694,27 @@
       </c>
       <c r="B17" s="8">
         <f>F16</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C17" s="8">
         <f>IF(A17&lt;=Supuestos!$B$15,B17*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D17" s="8">
         <f>E17-C17</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E17" s="8">
         <f>IF(A17&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F17" s="8">
         <f>B17-D17</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1636,22 +1724,27 @@
       </c>
       <c r="B18" s="12">
         <f>F17</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C18" s="12">
         <f>IF(A18&lt;=Supuestos!$B$15,B18*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D18" s="12">
         <f>E18-C18</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E18" s="12">
         <f>IF(A18&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F18" s="12">
         <f>B18-D18</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1661,22 +1754,27 @@
       </c>
       <c r="B19" s="8">
         <f>F18</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C19" s="8">
         <f>IF(A19&lt;=Supuestos!$B$15,B19*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D19" s="8">
         <f>E19-C19</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E19" s="8">
         <f>IF(A19&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F19" s="8">
         <f>B19-D19</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1686,22 +1784,27 @@
       </c>
       <c r="B20" s="12">
         <f>F19</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C20" s="12">
         <f>IF(A20&lt;=Supuestos!$B$15,B20*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D20" s="12">
         <f>E20-C20</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E20" s="12">
         <f>IF(A20&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F20" s="12">
         <f>B20-D20</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1711,22 +1814,27 @@
       </c>
       <c r="B21" s="8">
         <f>F20</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C21" s="8">
         <f>IF(A21&lt;=Supuestos!$B$15,B21*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D21" s="8">
         <f>E21-C21</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E21" s="8">
         <f>IF(A21&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F21" s="8">
         <f>B21-D21</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1736,22 +1844,27 @@
       </c>
       <c r="B22" s="12">
         <f>F21</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C22" s="12">
         <f>IF(A22&lt;=Supuestos!$B$15,B22*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D22" s="12">
         <f>E22-C22</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E22" s="12">
         <f>IF(A22&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F22" s="12">
         <f>B22-D22</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1761,22 +1874,27 @@
       </c>
       <c r="B23" s="8">
         <f>F22</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C23" s="8">
         <f>IF(A23&lt;=Supuestos!$B$15,B23*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D23" s="8">
         <f>E23-C23</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E23" s="8">
         <f>IF(A23&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F23" s="8">
         <f>B23-D23</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1786,22 +1904,27 @@
       </c>
       <c r="B24" s="12">
         <f>F23</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C24" s="12">
         <f>IF(A24&lt;=Supuestos!$B$15,B24*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D24" s="12">
         <f>E24-C24</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E24" s="12">
         <f>IF(A24&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F24" s="12">
         <f>B24-D24</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1811,22 +1934,27 @@
       </c>
       <c r="B25" s="8">
         <f>F24</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C25" s="8">
         <f>IF(A25&lt;=Supuestos!$B$15,B25*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D25" s="8">
         <f>E25-C25</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E25" s="8">
         <f>IF(A25&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F25" s="8">
         <f>B25-D25</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1836,22 +1964,27 @@
       </c>
       <c r="B26" s="12">
         <f>F25</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C26" s="12">
         <f>IF(A26&lt;=Supuestos!$B$15,B26*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D26" s="12">
         <f>E26-C26</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E26" s="12">
         <f>IF(A26&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F26" s="12">
         <f>B26-D26</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -1861,22 +1994,27 @@
       </c>
       <c r="B27" s="8">
         <f>F26</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="C27" s="8">
         <f>IF(A27&lt;=Supuestos!$B$15,B27*Supuestos!$B$11,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="D27" s="8">
         <f>E27-C27</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="E27" s="8">
         <f>IF(A27&lt;=Supuestos!$B$15,Supuestos!$B$24,0)</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="F27" s="8">
         <f>B27-D27</f>
+        <v>0.0</v>
         <v/>
       </c>
     </row>
@@ -2007,6 +2145,7 @@
       </c>
       <c r="K3" s="8">
         <f>Supuestos!$B$9</f>
+        <v>1997.1</v>
         <v/>
       </c>
       <c r="L3" s="8" t="n"/>
@@ -2021,50 +2160,62 @@
       </c>
       <c r="B4" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A4-1)</f>
+        <v>1500.0</v>
         <v/>
       </c>
       <c r="C4" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A4-1)</f>
+        <v>1150.0</v>
         <v/>
       </c>
       <c r="D4" s="8">
         <f>B4-C4</f>
+        <v>350.0</v>
         <v/>
       </c>
       <c r="E4" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F4" s="8">
         <f>D4-E4</f>
+        <v>-448.84</v>
         <v/>
       </c>
       <c r="G4" s="8">
         <f>'Amortizacion Deuda'!C3</f>
+        <v>219.681</v>
         <v/>
       </c>
       <c r="H4" s="8">
         <f>D4-MAX(F4,0)*Supuestos!$B$14</f>
+        <v>350.0</v>
         <v/>
       </c>
       <c r="I4" s="8">
         <f>(F4-G4)-MAX(F4-G4,0)*Supuestos!$B$14</f>
+        <v>-668.521</v>
         <v/>
       </c>
       <c r="J4" s="8">
         <f>I4+E4-'Amortizacion Deuda'!D3</f>
+        <v>10.88957</v>
         <v/>
       </c>
       <c r="K4" s="8">
         <f>-'Amortizacion Deuda'!E3</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L4" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A4-1)</f>
+        <v>4150.0</v>
         <v/>
       </c>
       <c r="M4" s="8">
         <f>L4-C4</f>
+        <v>3000.0</v>
         <v/>
       </c>
     </row>
@@ -2074,50 +2225,62 @@
       </c>
       <c r="B5" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A5-1)</f>
+        <v>1552.5</v>
         <v/>
       </c>
       <c r="C5" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A5-1)</f>
+        <v>1190.25</v>
         <v/>
       </c>
       <c r="D5" s="12">
         <f>B5-C5</f>
+        <v>362.25</v>
         <v/>
       </c>
       <c r="E5" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F5" s="12">
         <f>D5-E5</f>
+        <v>-436.59</v>
         <v/>
       </c>
       <c r="G5" s="12">
         <f>'Amortizacion Deuda'!C4</f>
+        <v>206.543763</v>
         <v/>
       </c>
       <c r="H5" s="12">
         <f>D5-MAX(F5,0)*Supuestos!$B$14</f>
+        <v>362.25</v>
         <v/>
       </c>
       <c r="I5" s="12">
         <f>(F5-G5)-MAX(F5-G5,0)*Supuestos!$B$14</f>
+        <v>-643.133763</v>
         <v/>
       </c>
       <c r="J5" s="12">
         <f>I5+E5-'Amortizacion Deuda'!D4</f>
+        <v>23.13957</v>
         <v/>
       </c>
       <c r="K5" s="12">
         <f>-'Amortizacion Deuda'!E4</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L5" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A5-1)</f>
+        <v>4295.25</v>
         <v/>
       </c>
       <c r="M5" s="12">
         <f>L5-C5</f>
+        <v>3105.0</v>
         <v/>
       </c>
     </row>
@@ -2127,50 +2290,62 @@
       </c>
       <c r="B6" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A6-1)</f>
+        <v>1606.8375</v>
         <v/>
       </c>
       <c r="C6" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A6-1)</f>
+        <v>1231.90875</v>
         <v/>
       </c>
       <c r="D6" s="8">
         <f>B6-C6</f>
+        <v>374.92875</v>
         <v/>
       </c>
       <c r="E6" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F6" s="8">
         <f>D6-E6</f>
+        <v>-423.91125</v>
         <v/>
       </c>
       <c r="G6" s="8">
         <f>'Amortizacion Deuda'!C5</f>
+        <v>191.961429</v>
         <v/>
       </c>
       <c r="H6" s="8">
         <f>D6-MAX(F6,0)*Supuestos!$B$14</f>
+        <v>374.92875</v>
         <v/>
       </c>
       <c r="I6" s="8">
         <f>(F6-G6)-MAX(F6-G6,0)*Supuestos!$B$14</f>
+        <v>-615.872679</v>
         <v/>
       </c>
       <c r="J6" s="8">
         <f>I6+E6-'Amortizacion Deuda'!D5</f>
+        <v>35.81832</v>
         <v/>
       </c>
       <c r="K6" s="8">
         <f>-'Amortizacion Deuda'!E5</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L6" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A6-1)</f>
+        <v>4445.58375</v>
         <v/>
       </c>
       <c r="M6" s="8">
         <f>L6-C6</f>
+        <v>3213.675</v>
         <v/>
       </c>
     </row>
@@ -2180,50 +2355,62 @@
       </c>
       <c r="B7" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A7-1)</f>
+        <v>1663.076812</v>
         <v/>
       </c>
       <c r="C7" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A7-1)</f>
+        <v>1275.025556</v>
         <v/>
       </c>
       <c r="D7" s="12">
         <f>B7-C7</f>
+        <v>388.051256</v>
         <v/>
       </c>
       <c r="E7" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F7" s="12">
         <f>D7-E7</f>
+        <v>-410.788744</v>
         <v/>
       </c>
       <c r="G7" s="12">
         <f>'Amortizacion Deuda'!C6</f>
+        <v>175.775039</v>
         <v/>
       </c>
       <c r="H7" s="12">
         <f>D7-MAX(F7,0)*Supuestos!$B$14</f>
+        <v>388.051256</v>
         <v/>
       </c>
       <c r="I7" s="12">
         <f>(F7-G7)-MAX(F7-G7,0)*Supuestos!$B$14</f>
+        <v>-586.563783</v>
         <v/>
       </c>
       <c r="J7" s="12">
         <f>I7+E7-'Amortizacion Deuda'!D6</f>
+        <v>48.940826</v>
         <v/>
       </c>
       <c r="K7" s="12">
         <f>-'Amortizacion Deuda'!E6</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L7" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A7-1)</f>
+        <v>4601.179181</v>
         <v/>
       </c>
       <c r="M7" s="12">
         <f>L7-C7</f>
+        <v>3326.153625</v>
         <v/>
       </c>
     </row>
@@ -2233,50 +2420,62 @@
       </c>
       <c r="B8" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A8-1)</f>
+        <v>1721.284501</v>
         <v/>
       </c>
       <c r="C8" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A8-1)</f>
+        <v>1319.651451</v>
         <v/>
       </c>
       <c r="D8" s="8">
         <f>B8-C8</f>
+        <v>401.63305</v>
         <v/>
       </c>
       <c r="E8" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F8" s="8">
         <f>D8-E8</f>
+        <v>-397.20695</v>
         <v/>
       </c>
       <c r="G8" s="8">
         <f>'Amortizacion Deuda'!C7</f>
+        <v>157.808146</v>
         <v/>
       </c>
       <c r="H8" s="8">
         <f>D8-MAX(F8,0)*Supuestos!$B$14</f>
+        <v>401.63305</v>
         <v/>
       </c>
       <c r="I8" s="8">
         <f>(F8-G8)-MAX(F8-G8,0)*Supuestos!$B$14</f>
+        <v>-555.015096</v>
         <v/>
       </c>
       <c r="J8" s="8">
         <f>I8+E8-'Amortizacion Deuda'!D7</f>
+        <v>62.52262</v>
         <v/>
       </c>
       <c r="K8" s="8">
         <f>-'Amortizacion Deuda'!E7</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L8" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A8-1)</f>
+        <v>4762.220453</v>
         <v/>
       </c>
       <c r="M8" s="8">
         <f>L8-C8</f>
+        <v>3442.569002</v>
         <v/>
       </c>
     </row>
@@ -2286,50 +2485,62 @@
       </c>
       <c r="B9" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A9-1)</f>
+        <v>1781.529458</v>
         <v/>
       </c>
       <c r="C9" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A9-1)</f>
+        <v>1365.839251</v>
         <v/>
       </c>
       <c r="D9" s="12">
         <f>B9-C9</f>
+        <v>415.690207</v>
         <v/>
       </c>
       <c r="E9" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F9" s="12">
         <f>D9-E9</f>
+        <v>-383.149793</v>
         <v/>
       </c>
       <c r="G9" s="12">
         <f>'Amortizacion Deuda'!C8</f>
+        <v>137.864895</v>
         <v/>
       </c>
       <c r="H9" s="12">
         <f>D9-MAX(F9,0)*Supuestos!$B$14</f>
+        <v>415.690207</v>
         <v/>
       </c>
       <c r="I9" s="12">
         <f>(F9-G9)-MAX(F9-G9,0)*Supuestos!$B$14</f>
+        <v>-521.014688</v>
         <v/>
       </c>
       <c r="J9" s="12">
         <f>I9+E9-'Amortizacion Deuda'!D8</f>
+        <v>76.579777</v>
         <v/>
       </c>
       <c r="K9" s="12">
         <f>-'Amortizacion Deuda'!E8</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L9" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A9-1)</f>
+        <v>4928.898168</v>
         <v/>
       </c>
       <c r="M9" s="12">
         <f>L9-C9</f>
+        <v>3563.058917</v>
         <v/>
       </c>
     </row>
@@ -2339,50 +2550,62 @@
       </c>
       <c r="B10" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A10-1)</f>
+        <v>1843.88299</v>
         <v/>
       </c>
       <c r="C10" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A10-1)</f>
+        <v>1413.643625</v>
         <v/>
       </c>
       <c r="D10" s="8">
         <f>B10-C10</f>
+        <v>430.239364</v>
         <v/>
       </c>
       <c r="E10" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F10" s="8">
         <f>D10-E10</f>
+        <v>-368.600636</v>
         <v/>
       </c>
       <c r="G10" s="8">
         <f>'Amortizacion Deuda'!C9</f>
+        <v>115.727886</v>
         <v/>
       </c>
       <c r="H10" s="8">
         <f>D10-MAX(F10,0)*Supuestos!$B$14</f>
+        <v>430.239364</v>
         <v/>
       </c>
       <c r="I10" s="8">
         <f>(F10-G10)-MAX(F10-G10,0)*Supuestos!$B$14</f>
+        <v>-484.328522</v>
         <v/>
       </c>
       <c r="J10" s="8">
         <f>I10+E10-'Amortizacion Deuda'!D9</f>
+        <v>91.128934</v>
         <v/>
       </c>
       <c r="K10" s="8">
         <f>-'Amortizacion Deuda'!E9</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L10" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A10-1)</f>
+        <v>5101.409604</v>
         <v/>
       </c>
       <c r="M10" s="8">
         <f>L10-C10</f>
+        <v>3687.765979</v>
         <v/>
       </c>
     </row>
@@ -2392,50 +2615,62 @@
       </c>
       <c r="B11" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A11-1)</f>
+        <v>1908.418894</v>
         <v/>
       </c>
       <c r="C11" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A11-1)</f>
+        <v>1463.121152</v>
         <v/>
       </c>
       <c r="D11" s="12">
         <f>B11-C11</f>
+        <v>445.297742</v>
         <v/>
       </c>
       <c r="E11" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F11" s="12">
         <f>D11-E11</f>
+        <v>-353.542258</v>
         <v/>
       </c>
       <c r="G11" s="12">
         <f>'Amortizacion Deuda'!C10</f>
+        <v>91.155806</v>
         <v/>
       </c>
       <c r="H11" s="12">
         <f>D11-MAX(F11,0)*Supuestos!$B$14</f>
+        <v>445.297742</v>
         <v/>
       </c>
       <c r="I11" s="12">
         <f>(F11-G11)-MAX(F11-G11,0)*Supuestos!$B$14</f>
+        <v>-444.698064</v>
         <v/>
       </c>
       <c r="J11" s="12">
         <f>I11+E11-'Amortizacion Deuda'!D10</f>
+        <v>106.187312</v>
         <v/>
       </c>
       <c r="K11" s="12">
         <f>-'Amortizacion Deuda'!E10</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L11" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A11-1)</f>
+        <v>5279.95894</v>
         <v/>
       </c>
       <c r="M11" s="12">
         <f>L11-C11</f>
+        <v>3816.837788</v>
         <v/>
       </c>
     </row>
@@ -2445,50 +2680,62 @@
       </c>
       <c r="B12" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A12-1)</f>
+        <v>1975.213555</v>
         <v/>
       </c>
       <c r="C12" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A12-1)</f>
+        <v>1514.330393</v>
         <v/>
       </c>
       <c r="D12" s="8">
         <f>B12-C12</f>
+        <v>460.883163</v>
         <v/>
       </c>
       <c r="E12" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F12" s="8">
         <f>D12-E12</f>
+        <v>-337.956837</v>
         <v/>
       </c>
       <c r="G12" s="8">
         <f>'Amortizacion Deuda'!C11</f>
+        <v>63.880798</v>
         <v/>
       </c>
       <c r="H12" s="8">
         <f>D12-MAX(F12,0)*Supuestos!$B$14</f>
+        <v>460.883163</v>
         <v/>
       </c>
       <c r="I12" s="8">
         <f>(F12-G12)-MAX(F12-G12,0)*Supuestos!$B$14</f>
+        <v>-401.837635</v>
         <v/>
       </c>
       <c r="J12" s="8">
         <f>I12+E12-'Amortizacion Deuda'!D11</f>
+        <v>121.772733</v>
         <v/>
       </c>
       <c r="K12" s="8">
         <f>-'Amortizacion Deuda'!E11</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L12" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A12-1)</f>
+        <v>5464.757503</v>
         <v/>
       </c>
       <c r="M12" s="8">
         <f>L12-C12</f>
+        <v>3950.427111</v>
         <v/>
       </c>
     </row>
@@ -2498,50 +2745,62 @@
       </c>
       <c r="B13" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A13-1)</f>
+        <v>2044.34603</v>
         <v/>
       </c>
       <c r="C13" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A13-1)</f>
+        <v>1567.331956</v>
         <v/>
       </c>
       <c r="D13" s="12">
         <f>B13-C13</f>
+        <v>477.014074</v>
         <v/>
       </c>
       <c r="E13" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F13" s="12">
         <f>D13-E13</f>
+        <v>-321.825926</v>
         <v/>
       </c>
       <c r="G13" s="12">
         <f>'Amortizacion Deuda'!C12</f>
+        <v>33.605538</v>
         <v/>
       </c>
       <c r="H13" s="12">
         <f>D13-MAX(F13,0)*Supuestos!$B$14</f>
+        <v>477.014074</v>
         <v/>
       </c>
       <c r="I13" s="12">
         <f>(F13-G13)-MAX(F13-G13,0)*Supuestos!$B$14</f>
+        <v>-355.431464</v>
         <v/>
       </c>
       <c r="J13" s="12">
         <f>I13+E13-'Amortizacion Deuda'!D12</f>
+        <v>137.903644</v>
         <v/>
       </c>
       <c r="K13" s="12">
         <f>-'Amortizacion Deuda'!E12</f>
+        <v>-339.11043</v>
         <v/>
       </c>
       <c r="L13" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A13-1)</f>
+        <v>5656.024016</v>
         <v/>
       </c>
       <c r="M13" s="12">
         <f>L13-C13</f>
+        <v>4088.69206</v>
         <v/>
       </c>
     </row>
@@ -2551,50 +2810,62 @@
       </c>
       <c r="B14" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A14-1)</f>
+        <v>2115.898141</v>
         <v/>
       </c>
       <c r="C14" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A14-1)</f>
+        <v>1622.188575</v>
         <v/>
       </c>
       <c r="D14" s="8">
         <f>B14-C14</f>
+        <v>493.709566</v>
         <v/>
       </c>
       <c r="E14" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F14" s="8">
         <f>D14-E14</f>
+        <v>-305.130434</v>
         <v/>
       </c>
       <c r="G14" s="8">
         <f>'Amortizacion Deuda'!C13</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H14" s="8">
         <f>D14-MAX(F14,0)*Supuestos!$B$14</f>
+        <v>493.709566</v>
         <v/>
       </c>
       <c r="I14" s="8">
         <f>(F14-G14)-MAX(F14-G14,0)*Supuestos!$B$14</f>
+        <v>-305.130434</v>
         <v/>
       </c>
       <c r="J14" s="8">
         <f>I14+E14-'Amortizacion Deuda'!D13</f>
+        <v>493.709566</v>
         <v/>
       </c>
       <c r="K14" s="8">
         <f>-'Amortizacion Deuda'!E13</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L14" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A14-1)</f>
+        <v>5853.984857</v>
         <v/>
       </c>
       <c r="M14" s="8">
         <f>L14-C14</f>
+        <v>4231.796282</v>
         <v/>
       </c>
     </row>
@@ -2604,50 +2875,62 @@
       </c>
       <c r="B15" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A15-1)</f>
+        <v>2189.954576</v>
         <v/>
       </c>
       <c r="C15" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A15-1)</f>
+        <v>1678.965175</v>
         <v/>
       </c>
       <c r="D15" s="12">
         <f>B15-C15</f>
+        <v>510.989401</v>
         <v/>
       </c>
       <c r="E15" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F15" s="12">
         <f>D15-E15</f>
+        <v>-287.850599</v>
         <v/>
       </c>
       <c r="G15" s="12">
         <f>'Amortizacion Deuda'!C14</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H15" s="12">
         <f>D15-MAX(F15,0)*Supuestos!$B$14</f>
+        <v>510.989401</v>
         <v/>
       </c>
       <c r="I15" s="12">
         <f>(F15-G15)-MAX(F15-G15,0)*Supuestos!$B$14</f>
+        <v>-287.850599</v>
         <v/>
       </c>
       <c r="J15" s="12">
         <f>I15+E15-'Amortizacion Deuda'!D14</f>
+        <v>510.989401</v>
         <v/>
       </c>
       <c r="K15" s="12">
         <f>-'Amortizacion Deuda'!E14</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L15" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A15-1)</f>
+        <v>6058.874327</v>
         <v/>
       </c>
       <c r="M15" s="12">
         <f>L15-C15</f>
+        <v>4379.909152</v>
         <v/>
       </c>
     </row>
@@ -2657,50 +2940,62 @@
       </c>
       <c r="B16" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A16-1)</f>
+        <v>2266.602986</v>
         <v/>
       </c>
       <c r="C16" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A16-1)</f>
+        <v>1737.728956</v>
         <v/>
       </c>
       <c r="D16" s="8">
         <f>B16-C16</f>
+        <v>528.87403</v>
         <v/>
       </c>
       <c r="E16" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F16" s="8">
         <f>D16-E16</f>
+        <v>-269.96597</v>
         <v/>
       </c>
       <c r="G16" s="8">
         <f>'Amortizacion Deuda'!C15</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H16" s="8">
         <f>D16-MAX(F16,0)*Supuestos!$B$14</f>
+        <v>528.87403</v>
         <v/>
       </c>
       <c r="I16" s="8">
         <f>(F16-G16)-MAX(F16-G16,0)*Supuestos!$B$14</f>
+        <v>-269.96597</v>
         <v/>
       </c>
       <c r="J16" s="8">
         <f>I16+E16-'Amortizacion Deuda'!D15</f>
+        <v>528.87403</v>
         <v/>
       </c>
       <c r="K16" s="8">
         <f>-'Amortizacion Deuda'!E15</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L16" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A16-1)</f>
+        <v>6270.934928</v>
         <v/>
       </c>
       <c r="M16" s="8">
         <f>L16-C16</f>
+        <v>4533.205972</v>
         <v/>
       </c>
     </row>
@@ -2710,50 +3005,62 @@
       </c>
       <c r="B17" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A17-1)</f>
+        <v>2345.934091</v>
         <v/>
       </c>
       <c r="C17" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A17-1)</f>
+        <v>1798.549469</v>
         <v/>
       </c>
       <c r="D17" s="12">
         <f>B17-C17</f>
+        <v>547.384621</v>
         <v/>
       </c>
       <c r="E17" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F17" s="12">
         <f>D17-E17</f>
+        <v>-251.455379</v>
         <v/>
       </c>
       <c r="G17" s="12">
         <f>'Amortizacion Deuda'!C16</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H17" s="12">
         <f>D17-MAX(F17,0)*Supuestos!$B$14</f>
+        <v>547.384621</v>
         <v/>
       </c>
       <c r="I17" s="12">
         <f>(F17-G17)-MAX(F17-G17,0)*Supuestos!$B$14</f>
+        <v>-251.455379</v>
         <v/>
       </c>
       <c r="J17" s="12">
         <f>I17+E17-'Amortizacion Deuda'!D16</f>
+        <v>547.384621</v>
         <v/>
       </c>
       <c r="K17" s="12">
         <f>-'Amortizacion Deuda'!E16</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L17" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A17-1)</f>
+        <v>6490.41765</v>
         <v/>
       </c>
       <c r="M17" s="12">
         <f>L17-C17</f>
+        <v>4691.868181</v>
         <v/>
       </c>
     </row>
@@ -2763,50 +3070,62 @@
       </c>
       <c r="B18" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A18-1)</f>
+        <v>2428.041784</v>
         <v/>
       </c>
       <c r="C18" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A18-1)</f>
+        <v>1861.498701</v>
         <v/>
       </c>
       <c r="D18" s="8">
         <f>B18-C18</f>
+        <v>566.543083</v>
         <v/>
       </c>
       <c r="E18" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F18" s="8">
         <f>D18-E18</f>
+        <v>-232.296917</v>
         <v/>
       </c>
       <c r="G18" s="8">
         <f>'Amortizacion Deuda'!C17</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H18" s="8">
         <f>D18-MAX(F18,0)*Supuestos!$B$14</f>
+        <v>566.543083</v>
         <v/>
       </c>
       <c r="I18" s="8">
         <f>(F18-G18)-MAX(F18-G18,0)*Supuestos!$B$14</f>
+        <v>-232.296917</v>
         <v/>
       </c>
       <c r="J18" s="8">
         <f>I18+E18-'Amortizacion Deuda'!D17</f>
+        <v>566.543083</v>
         <v/>
       </c>
       <c r="K18" s="8">
         <f>-'Amortizacion Deuda'!E17</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L18" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A18-1)</f>
+        <v>6717.582268</v>
         <v/>
       </c>
       <c r="M18" s="8">
         <f>L18-C18</f>
+        <v>4856.083567</v>
         <v/>
       </c>
     </row>
@@ -2816,50 +3135,62 @@
       </c>
       <c r="B19" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A19-1)</f>
+        <v>2513.023246</v>
         <v/>
       </c>
       <c r="C19" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A19-1)</f>
+        <v>1926.651155</v>
         <v/>
       </c>
       <c r="D19" s="12">
         <f>B19-C19</f>
+        <v>586.372091</v>
         <v/>
       </c>
       <c r="E19" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F19" s="12">
         <f>D19-E19</f>
+        <v>-212.467909</v>
         <v/>
       </c>
       <c r="G19" s="12">
         <f>'Amortizacion Deuda'!C18</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H19" s="12">
         <f>D19-MAX(F19,0)*Supuestos!$B$14</f>
+        <v>586.372091</v>
         <v/>
       </c>
       <c r="I19" s="12">
         <f>(F19-G19)-MAX(F19-G19,0)*Supuestos!$B$14</f>
+        <v>-212.467909</v>
         <v/>
       </c>
       <c r="J19" s="12">
         <f>I19+E19-'Amortizacion Deuda'!D18</f>
+        <v>586.372091</v>
         <v/>
       </c>
       <c r="K19" s="12">
         <f>-'Amortizacion Deuda'!E18</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L19" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A19-1)</f>
+        <v>6952.697648</v>
         <v/>
       </c>
       <c r="M19" s="12">
         <f>L19-C19</f>
+        <v>5026.046492</v>
         <v/>
       </c>
     </row>
@@ -2869,50 +3200,62 @@
       </c>
       <c r="B20" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A20-1)</f>
+        <v>2600.97906</v>
         <v/>
       </c>
       <c r="C20" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A20-1)</f>
+        <v>1994.083946</v>
         <v/>
       </c>
       <c r="D20" s="8">
         <f>B20-C20</f>
+        <v>606.895114</v>
         <v/>
       </c>
       <c r="E20" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F20" s="8">
         <f>D20-E20</f>
+        <v>-191.944886</v>
         <v/>
       </c>
       <c r="G20" s="8">
         <f>'Amortizacion Deuda'!C19</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H20" s="8">
         <f>D20-MAX(F20,0)*Supuestos!$B$14</f>
+        <v>606.895114</v>
         <v/>
       </c>
       <c r="I20" s="8">
         <f>(F20-G20)-MAX(F20-G20,0)*Supuestos!$B$14</f>
+        <v>-191.944886</v>
         <v/>
       </c>
       <c r="J20" s="8">
         <f>I20+E20-'Amortizacion Deuda'!D19</f>
+        <v>606.895114</v>
         <v/>
       </c>
       <c r="K20" s="8">
         <f>-'Amortizacion Deuda'!E19</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L20" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A20-1)</f>
+        <v>7196.042065</v>
         <v/>
       </c>
       <c r="M20" s="8">
         <f>L20-C20</f>
+        <v>5201.958119</v>
         <v/>
       </c>
     </row>
@@ -2922,50 +3265,62 @@
       </c>
       <c r="B21" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A21-1)</f>
+        <v>2692.013327</v>
         <v/>
       </c>
       <c r="C21" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A21-1)</f>
+        <v>2063.876884</v>
         <v/>
       </c>
       <c r="D21" s="12">
         <f>B21-C21</f>
+        <v>628.136443</v>
         <v/>
       </c>
       <c r="E21" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F21" s="12">
         <f>D21-E21</f>
+        <v>-170.703557</v>
         <v/>
       </c>
       <c r="G21" s="12">
         <f>'Amortizacion Deuda'!C20</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H21" s="12">
         <f>D21-MAX(F21,0)*Supuestos!$B$14</f>
+        <v>628.136443</v>
         <v/>
       </c>
       <c r="I21" s="12">
         <f>(F21-G21)-MAX(F21-G21,0)*Supuestos!$B$14</f>
+        <v>-170.703557</v>
         <v/>
       </c>
       <c r="J21" s="12">
         <f>I21+E21-'Amortizacion Deuda'!D20</f>
+        <v>628.136443</v>
         <v/>
       </c>
       <c r="K21" s="12">
         <f>-'Amortizacion Deuda'!E20</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L21" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A21-1)</f>
+        <v>7447.903538</v>
         <v/>
       </c>
       <c r="M21" s="12">
         <f>L21-C21</f>
+        <v>5384.026654</v>
         <v/>
       </c>
     </row>
@@ -2975,50 +3330,62 @@
       </c>
       <c r="B22" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A22-1)</f>
+        <v>2786.233793</v>
         <v/>
       </c>
       <c r="C22" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A22-1)</f>
+        <v>2136.112575</v>
         <v/>
       </c>
       <c r="D22" s="8">
         <f>B22-C22</f>
+        <v>650.121218</v>
         <v/>
       </c>
       <c r="E22" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F22" s="8">
         <f>D22-E22</f>
+        <v>-148.718782</v>
         <v/>
       </c>
       <c r="G22" s="8">
         <f>'Amortizacion Deuda'!C21</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H22" s="8">
         <f>D22-MAX(F22,0)*Supuestos!$B$14</f>
+        <v>650.121218</v>
         <v/>
       </c>
       <c r="I22" s="8">
         <f>(F22-G22)-MAX(F22-G22,0)*Supuestos!$B$14</f>
+        <v>-148.718782</v>
         <v/>
       </c>
       <c r="J22" s="8">
         <f>I22+E22-'Amortizacion Deuda'!D21</f>
+        <v>650.121218</v>
         <v/>
       </c>
       <c r="K22" s="8">
         <f>-'Amortizacion Deuda'!E21</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L22" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A22-1)</f>
+        <v>7708.580161</v>
         <v/>
       </c>
       <c r="M22" s="8">
         <f>L22-C22</f>
+        <v>5572.467587</v>
         <v/>
       </c>
     </row>
@@ -3028,50 +3395,62 @@
       </c>
       <c r="B23" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A23-1)</f>
+        <v>2883.751976</v>
         <v/>
       </c>
       <c r="C23" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A23-1)</f>
+        <v>2210.876515</v>
         <v/>
       </c>
       <c r="D23" s="12">
         <f>B23-C23</f>
+        <v>672.875461</v>
         <v/>
       </c>
       <c r="E23" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F23" s="12">
         <f>D23-E23</f>
+        <v>-125.964539</v>
         <v/>
       </c>
       <c r="G23" s="12">
         <f>'Amortizacion Deuda'!C22</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H23" s="12">
         <f>D23-MAX(F23,0)*Supuestos!$B$14</f>
+        <v>672.875461</v>
         <v/>
       </c>
       <c r="I23" s="12">
         <f>(F23-G23)-MAX(F23-G23,0)*Supuestos!$B$14</f>
+        <v>-125.964539</v>
         <v/>
       </c>
       <c r="J23" s="12">
         <f>I23+E23-'Amortizacion Deuda'!D22</f>
+        <v>672.875461</v>
         <v/>
       </c>
       <c r="K23" s="12">
         <f>-'Amortizacion Deuda'!E22</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L23" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A23-1)</f>
+        <v>7978.380467</v>
         <v/>
       </c>
       <c r="M23" s="12">
         <f>L23-C23</f>
+        <v>5767.503952</v>
         <v/>
       </c>
     </row>
@@ -3081,50 +3460,62 @@
       </c>
       <c r="B24" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A24-1)</f>
+        <v>2984.683295</v>
         <v/>
       </c>
       <c r="C24" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A24-1)</f>
+        <v>2288.257193</v>
         <v/>
       </c>
       <c r="D24" s="8">
         <f>B24-C24</f>
+        <v>696.426102</v>
         <v/>
       </c>
       <c r="E24" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F24" s="8">
         <f>D24-E24</f>
+        <v>-102.413898</v>
         <v/>
       </c>
       <c r="G24" s="8">
         <f>'Amortizacion Deuda'!C23</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H24" s="8">
         <f>D24-MAX(F24,0)*Supuestos!$B$14</f>
+        <v>696.426102</v>
         <v/>
       </c>
       <c r="I24" s="8">
         <f>(F24-G24)-MAX(F24-G24,0)*Supuestos!$B$14</f>
+        <v>-102.413898</v>
         <v/>
       </c>
       <c r="J24" s="8">
         <f>I24+E24-'Amortizacion Deuda'!D23</f>
+        <v>696.426102</v>
         <v/>
       </c>
       <c r="K24" s="8">
         <f>-'Amortizacion Deuda'!E23</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L24" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A24-1)</f>
+        <v>8257.623783</v>
         <v/>
       </c>
       <c r="M24" s="8">
         <f>L24-C24</f>
+        <v>5969.36659</v>
         <v/>
       </c>
     </row>
@@ -3134,50 +3525,62 @@
       </c>
       <c r="B25" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A25-1)</f>
+        <v>3089.147211</v>
         <v/>
       </c>
       <c r="C25" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A25-1)</f>
+        <v>2368.346195</v>
         <v/>
       </c>
       <c r="D25" s="12">
         <f>B25-C25</f>
+        <v>720.801016</v>
         <v/>
       </c>
       <c r="E25" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F25" s="12">
         <f>D25-E25</f>
+        <v>-78.038984</v>
         <v/>
       </c>
       <c r="G25" s="12">
         <f>'Amortizacion Deuda'!C24</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H25" s="12">
         <f>D25-MAX(F25,0)*Supuestos!$B$14</f>
+        <v>720.801016</v>
         <v/>
       </c>
       <c r="I25" s="12">
         <f>(F25-G25)-MAX(F25-G25,0)*Supuestos!$B$14</f>
+        <v>-78.038984</v>
         <v/>
       </c>
       <c r="J25" s="12">
         <f>I25+E25-'Amortizacion Deuda'!D24</f>
+        <v>720.801016</v>
         <v/>
       </c>
       <c r="K25" s="12">
         <f>-'Amortizacion Deuda'!E24</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L25" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A25-1)</f>
+        <v>8546.640616</v>
         <v/>
       </c>
       <c r="M25" s="12">
         <f>L25-C25</f>
+        <v>6178.294421</v>
         <v/>
       </c>
     </row>
@@ -3187,50 +3590,62 @@
       </c>
       <c r="B26" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A26-1)</f>
+        <v>3197.267363</v>
         <v/>
       </c>
       <c r="C26" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A26-1)</f>
+        <v>2451.238312</v>
         <v/>
       </c>
       <c r="D26" s="8">
         <f>B26-C26</f>
+        <v>746.029051</v>
         <v/>
       </c>
       <c r="E26" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F26" s="8">
         <f>D26-E26</f>
+        <v>-52.810949</v>
         <v/>
       </c>
       <c r="G26" s="8">
         <f>'Amortizacion Deuda'!C25</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H26" s="8">
         <f>D26-MAX(F26,0)*Supuestos!$B$14</f>
+        <v>746.029051</v>
         <v/>
       </c>
       <c r="I26" s="8">
         <f>(F26-G26)-MAX(F26-G26,0)*Supuestos!$B$14</f>
+        <v>-52.810949</v>
         <v/>
       </c>
       <c r="J26" s="8">
         <f>I26+E26-'Amortizacion Deuda'!D25</f>
+        <v>746.029051</v>
         <v/>
       </c>
       <c r="K26" s="8">
         <f>-'Amortizacion Deuda'!E25</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L26" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A26-1)</f>
+        <v>8845.773037</v>
         <v/>
       </c>
       <c r="M26" s="8">
         <f>L26-C26</f>
+        <v>6394.534726</v>
         <v/>
       </c>
     </row>
@@ -3240,50 +3655,62 @@
       </c>
       <c r="B27" s="12">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A27-1)</f>
+        <v>3309.171721</v>
         <v/>
       </c>
       <c r="C27" s="12">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A27-1)</f>
+        <v>2537.031652</v>
         <v/>
       </c>
       <c r="D27" s="12">
         <f>B27-C27</f>
+        <v>772.140068</v>
         <v/>
       </c>
       <c r="E27" s="12">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F27" s="12">
         <f>D27-E27</f>
+        <v>-26.699932</v>
         <v/>
       </c>
       <c r="G27" s="12">
         <f>'Amortizacion Deuda'!C26</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H27" s="12">
         <f>D27-MAX(F27,0)*Supuestos!$B$14</f>
+        <v>772.140068</v>
         <v/>
       </c>
       <c r="I27" s="12">
         <f>(F27-G27)-MAX(F27-G27,0)*Supuestos!$B$14</f>
+        <v>-26.699932</v>
         <v/>
       </c>
       <c r="J27" s="12">
         <f>I27+E27-'Amortizacion Deuda'!D26</f>
+        <v>772.140068</v>
         <v/>
       </c>
       <c r="K27" s="12">
         <f>-'Amortizacion Deuda'!E26</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L27" s="12">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A27-1)</f>
+        <v>9155.375094</v>
         <v/>
       </c>
       <c r="M27" s="12">
         <f>L27-C27</f>
+        <v>6618.343441</v>
         <v/>
       </c>
     </row>
@@ -3293,50 +3720,62 @@
       </c>
       <c r="B28" s="8">
         <f>Supuestos!$B$17*(1+Supuestos!$B$18)^(A28-1)</f>
+        <v>3424.992731</v>
         <v/>
       </c>
       <c r="C28" s="8">
         <f>Supuestos!$B$19*(1+Supuestos!$B$20)^(A28-1)</f>
+        <v>2625.82776</v>
         <v/>
       </c>
       <c r="D28" s="8">
         <f>B28-C28</f>
+        <v>799.164971</v>
         <v/>
       </c>
       <c r="E28" s="8">
         <f>Supuestos!$B$23</f>
+        <v>798.84</v>
         <v/>
       </c>
       <c r="F28" s="8">
         <f>D28-E28</f>
+        <v>0.324971</v>
         <v/>
       </c>
       <c r="G28" s="8">
         <f>'Amortizacion Deuda'!C27</f>
+        <v>0.0</v>
         <v/>
       </c>
       <c r="H28" s="8">
         <f>D28-MAX(F28,0)*Supuestos!$B$14</f>
+        <v>799.051231</v>
         <v/>
       </c>
       <c r="I28" s="8">
         <f>(F28-G28)-MAX(F28-G28,0)*Supuestos!$B$14</f>
+        <v>0.211231</v>
         <v/>
       </c>
       <c r="J28" s="8">
         <f>I28+E28-'Amortizacion Deuda'!D27</f>
+        <v>799.051231</v>
         <v/>
       </c>
       <c r="K28" s="8">
         <f>-'Amortizacion Deuda'!E27</f>
+        <v>-0.0</v>
         <v/>
       </c>
       <c r="L28" s="8">
         <f>Supuestos!$B$21*(1+Supuestos!$B$22)^(A28-1)</f>
+        <v>9475.813222</v>
         <v/>
       </c>
       <c r="M28" s="8">
         <f>L28-C28</f>
+        <v>6849.985462</v>
         <v/>
       </c>
     </row>
@@ -3394,6 +3833,7 @@
       </c>
       <c r="B3" s="13">
         <f>Supuestos!$B$25</f>
+        <v>0.09315</v>
         <v/>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -3410,6 +3850,7 @@
       </c>
       <c r="B4" s="13">
         <f>'Flujos de Caja'!$H$3+NPV(Supuestos!$B$25,'Flujos de Caja'!$H$4:$H$28)</f>
+        <v>-15486.829599</v>
         <v/>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -3426,6 +3867,7 @@
       </c>
       <c r="B5" s="13">
         <f>IRR('Flujos de Caja'!$H$3:$H$28)</f>
+        <v>-0.024526</v>
         <v/>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -3442,6 +3884,7 @@
       </c>
       <c r="B6" s="14">
         <f>'Flujos de Caja'!$J$3+NPV(Supuestos!$B$12,'Flujos de Caja'!$J$4:$J$28)</f>
+        <v>-730.301529</v>
         <v/>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -3458,6 +3901,7 @@
       </c>
       <c r="B7" s="13">
         <f>IRR('Flujos de Caja'!$J$3:$J$28)</f>
+        <v>0.104611</v>
         <v/>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -3474,6 +3918,7 @@
       </c>
       <c r="B8" s="14">
         <f>'Flujos de Caja'!$M$3+NPV(Supuestos!$B$13,'Flujos de Caja'!$M$4:$M$28)</f>
+        <v>19625.705143</v>
         <v/>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -3490,6 +3935,7 @@
       </c>
       <c r="B9" s="15">
         <f>NPV(Supuestos!$B$13,'Flujos de Caja'!$L$4:$L$28)/(Supuestos!$B$4+NPV(Supuestos!$B$13,'Flujos de Caja'!$C$4:$C$28))</f>
+        <v>1.558346</v>
         <v/>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -3591,10 +4037,12 @@
       </c>
       <c r="F3" s="9">
         <f>D3*E3</f>
-        <v/>
-      </c>
-      <c r="G3" s="9">
+        <v>20.0</v>
+        <v/>
+      </c>
+      <c r="G3" s="9" t="str">
         <f>IF(F3&gt;=15,"Alto",IF(F3&gt;=8,"Medio","Bajo"))</f>
+        <v>Alto</v>
         <v/>
       </c>
     </row>
@@ -3620,10 +4068,12 @@
       </c>
       <c r="F4" s="9">
         <f>D4*E4</f>
-        <v/>
-      </c>
-      <c r="G4" s="9">
+        <v>20.0</v>
+        <v/>
+      </c>
+      <c r="G4" s="9" t="str">
         <f>IF(F4&gt;=15,"Alto",IF(F4&gt;=8,"Medio","Bajo"))</f>
+        <v>Alto</v>
         <v/>
       </c>
     </row>
@@ -3649,10 +4099,12 @@
       </c>
       <c r="F5" s="9">
         <f>D5*E5</f>
-        <v/>
-      </c>
-      <c r="G5" s="9">
+        <v>16.0</v>
+        <v/>
+      </c>
+      <c r="G5" s="9" t="str">
         <f>IF(F5&gt;=15,"Alto",IF(F5&gt;=8,"Medio","Bajo"))</f>
+        <v>Alto</v>
         <v/>
       </c>
     </row>
@@ -3678,10 +4130,12 @@
       </c>
       <c r="F6" s="9">
         <f>D6*E6</f>
-        <v/>
-      </c>
-      <c r="G6" s="9">
+        <v>9.0</v>
+        <v/>
+      </c>
+      <c r="G6" s="9" t="str">
         <f>IF(F6&gt;=15,"Alto",IF(F6&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3707,10 +4161,12 @@
       </c>
       <c r="F7" s="9">
         <f>D7*E7</f>
-        <v/>
-      </c>
-      <c r="G7" s="9">
+        <v>12.0</v>
+        <v/>
+      </c>
+      <c r="G7" s="9" t="str">
         <f>IF(F7&gt;=15,"Alto",IF(F7&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3736,10 +4192,12 @@
       </c>
       <c r="F8" s="9">
         <f>D8*E8</f>
-        <v/>
-      </c>
-      <c r="G8" s="9">
+        <v>9.0</v>
+        <v/>
+      </c>
+      <c r="G8" s="9" t="str">
         <f>IF(F8&gt;=15,"Alto",IF(F8&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3765,10 +4223,12 @@
       </c>
       <c r="F9" s="9">
         <f>D9*E9</f>
-        <v/>
-      </c>
-      <c r="G9" s="9">
+        <v>12.0</v>
+        <v/>
+      </c>
+      <c r="G9" s="9" t="str">
         <f>IF(F9&gt;=15,"Alto",IF(F9&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3794,10 +4254,12 @@
       </c>
       <c r="F10" s="9">
         <f>D10*E10</f>
-        <v/>
-      </c>
-      <c r="G10" s="9">
+        <v>16.0</v>
+        <v/>
+      </c>
+      <c r="G10" s="9" t="str">
         <f>IF(F10&gt;=15,"Alto",IF(F10&gt;=8,"Medio","Bajo"))</f>
+        <v>Alto</v>
         <v/>
       </c>
     </row>
@@ -3823,10 +4285,12 @@
       </c>
       <c r="F11" s="9">
         <f>D11*E11</f>
-        <v/>
-      </c>
-      <c r="G11" s="9">
+        <v>16.0</v>
+        <v/>
+      </c>
+      <c r="G11" s="9" t="str">
         <f>IF(F11&gt;=15,"Alto",IF(F11&gt;=8,"Medio","Bajo"))</f>
+        <v>Alto</v>
         <v/>
       </c>
     </row>
@@ -3852,10 +4316,12 @@
       </c>
       <c r="F12" s="9">
         <f>D12*E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="9">
+        <v>12.0</v>
+        <v/>
+      </c>
+      <c r="G12" s="9" t="str">
         <f>IF(F12&gt;=15,"Alto",IF(F12&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3881,10 +4347,12 @@
       </c>
       <c r="F13" s="9">
         <f>D13*E13</f>
-        <v/>
-      </c>
-      <c r="G13" s="9">
+        <v>9.0</v>
+        <v/>
+      </c>
+      <c r="G13" s="9" t="str">
         <f>IF(F13&gt;=15,"Alto",IF(F13&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3910,10 +4378,12 @@
       </c>
       <c r="F14" s="9">
         <f>D14*E14</f>
-        <v/>
-      </c>
-      <c r="G14" s="9">
+        <v>12.0</v>
+        <v/>
+      </c>
+      <c r="G14" s="9" t="str">
         <f>IF(F14&gt;=15,"Alto",IF(F14&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3939,10 +4409,12 @@
       </c>
       <c r="F15" s="9">
         <f>D15*E15</f>
-        <v/>
-      </c>
-      <c r="G15" s="9">
+        <v>8.0</v>
+        <v/>
+      </c>
+      <c r="G15" s="9" t="str">
         <f>IF(F15&gt;=15,"Alto",IF(F15&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3968,10 +4440,12 @@
       </c>
       <c r="F16" s="9">
         <f>D16*E16</f>
-        <v/>
-      </c>
-      <c r="G16" s="9">
+        <v>9.0</v>
+        <v/>
+      </c>
+      <c r="G16" s="9" t="str">
         <f>IF(F16&gt;=15,"Alto",IF(F16&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -3997,10 +4471,12 @@
       </c>
       <c r="F17" s="9">
         <f>D17*E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="9">
+        <v>12.0</v>
+        <v/>
+      </c>
+      <c r="G17" s="9" t="str">
         <f>IF(F17&gt;=15,"Alto",IF(F17&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4026,10 +4502,12 @@
       </c>
       <c r="F18" s="9">
         <f>D18*E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="9">
+        <v>9.0</v>
+        <v/>
+      </c>
+      <c r="G18" s="9" t="str">
         <f>IF(F18&gt;=15,"Alto",IF(F18&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4055,10 +4533,12 @@
       </c>
       <c r="F19" s="9">
         <f>D19*E19</f>
-        <v/>
-      </c>
-      <c r="G19" s="9">
+        <v>12.0</v>
+        <v/>
+      </c>
+      <c r="G19" s="9" t="str">
         <f>IF(F19&gt;=15,"Alto",IF(F19&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4084,10 +4564,12 @@
       </c>
       <c r="F20" s="9">
         <f>D20*E20</f>
-        <v/>
-      </c>
-      <c r="G20" s="9">
+        <v>6.0</v>
+        <v/>
+      </c>
+      <c r="G20" s="9" t="str">
         <f>IF(F20&gt;=15,"Alto",IF(F20&gt;=8,"Medio","Bajo"))</f>
+        <v>Bajo</v>
         <v/>
       </c>
     </row>
@@ -4113,10 +4595,12 @@
       </c>
       <c r="F21" s="9">
         <f>D21*E21</f>
-        <v/>
-      </c>
-      <c r="G21" s="9">
+        <v>9.0</v>
+        <v/>
+      </c>
+      <c r="G21" s="9" t="str">
         <f>IF(F21&gt;=15,"Alto",IF(F21&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4142,10 +4626,12 @@
       </c>
       <c r="F22" s="9">
         <f>D22*E22</f>
-        <v/>
-      </c>
-      <c r="G22" s="9">
+        <v>8.0</v>
+        <v/>
+      </c>
+      <c r="G22" s="9" t="str">
         <f>IF(F22&gt;=15,"Alto",IF(F22&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4225,10 +4711,12 @@
       </c>
       <c r="G27" s="9">
         <f>E27*F27</f>
-        <v/>
-      </c>
-      <c r="H27" s="9">
+        <v>8.0</v>
+        <v/>
+      </c>
+      <c r="H27" s="9" t="str">
         <f>IF(G27&gt;=15,"Alto",IF(G27&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4259,10 +4747,12 @@
       </c>
       <c r="G28" s="9">
         <f>E28*F28</f>
-        <v/>
-      </c>
-      <c r="H28" s="9">
+        <v>9.0</v>
+        <v/>
+      </c>
+      <c r="H28" s="9" t="str">
         <f>IF(G28&gt;=15,"Alto",IF(G28&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4293,10 +4783,12 @@
       </c>
       <c r="G29" s="9">
         <f>E29*F29</f>
-        <v/>
-      </c>
-      <c r="H29" s="9">
+        <v>8.0</v>
+        <v/>
+      </c>
+      <c r="H29" s="9" t="str">
         <f>IF(G29&gt;=15,"Alto",IF(G29&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4327,10 +4819,12 @@
       </c>
       <c r="G30" s="9">
         <f>E30*F30</f>
-        <v/>
-      </c>
-      <c r="H30" s="9">
+        <v>6.0</v>
+        <v/>
+      </c>
+      <c r="H30" s="9" t="str">
         <f>IF(G30&gt;=15,"Alto",IF(G30&gt;=8,"Medio","Bajo"))</f>
+        <v>Bajo</v>
         <v/>
       </c>
     </row>
@@ -4361,10 +4855,12 @@
       </c>
       <c r="G31" s="9">
         <f>E31*F31</f>
-        <v/>
-      </c>
-      <c r="H31" s="9">
+        <v>4.0</v>
+        <v/>
+      </c>
+      <c r="H31" s="9" t="str">
         <f>IF(G31&gt;=15,"Alto",IF(G31&gt;=8,"Medio","Bajo"))</f>
+        <v>Bajo</v>
         <v/>
       </c>
     </row>
@@ -4395,10 +4891,12 @@
       </c>
       <c r="G32" s="9">
         <f>E32*F32</f>
-        <v/>
-      </c>
-      <c r="H32" s="9">
+        <v>8.0</v>
+        <v/>
+      </c>
+      <c r="H32" s="9" t="str">
         <f>IF(G32&gt;=15,"Alto",IF(G32&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4429,10 +4927,12 @@
       </c>
       <c r="G33" s="9">
         <f>E33*F33</f>
-        <v/>
-      </c>
-      <c r="H33" s="9">
+        <v>8.0</v>
+        <v/>
+      </c>
+      <c r="H33" s="9" t="str">
         <f>IF(G33&gt;=15,"Alto",IF(G33&gt;=8,"Medio","Bajo"))</f>
+        <v>Medio</v>
         <v/>
       </c>
     </row>
@@ -4463,10 +4963,12 @@
       </c>
       <c r="G34" s="9">
         <f>E34*F34</f>
-        <v/>
-      </c>
-      <c r="H34" s="9">
+        <v>6.0</v>
+        <v/>
+      </c>
+      <c r="H34" s="9" t="str">
         <f>IF(G34&gt;=15,"Alto",IF(G34&gt;=8,"Medio","Bajo"))</f>
+        <v>Bajo</v>
         <v/>
       </c>
     </row>
@@ -4497,10 +4999,12 @@
       </c>
       <c r="G35" s="9">
         <f>E35*F35</f>
-        <v/>
-      </c>
-      <c r="H35" s="9">
+        <v>6.0</v>
+        <v/>
+      </c>
+      <c r="H35" s="9" t="str">
         <f>IF(G35&gt;=15,"Alto",IF(G35&gt;=8,"Medio","Bajo"))</f>
+        <v>Bajo</v>
         <v/>
       </c>
     </row>
@@ -4531,10 +5035,12 @@
       </c>
       <c r="G36" s="9">
         <f>E36*F36</f>
-        <v/>
-      </c>
-      <c r="H36" s="9">
+        <v>6.0</v>
+        <v/>
+      </c>
+      <c r="H36" s="9" t="str">
         <f>IF(G36&gt;=15,"Alto",IF(G36&gt;=8,"Medio","Bajo"))</f>
+        <v>Bajo</v>
         <v/>
       </c>
     </row>

</xml_diff>